<commit_message>
Urgency: don't mark high on estimated-zero stock or rarely stocked items; demo free stock
- core: 'stock_uncertain' when zero comes from estimate (start-of-month stock > 0, no free-stock
  column) and 'rarely_stocked' when out of stock >=6 of 12 months — both cap urgency at medium,
  order quantity unchanged; notes added to rationale; UI flags
- demo data: 'Свободный остаток' column (actual simulated stock), like Systeme Electric
- IEK urgent share 42% -> 24%, Systeme Electric 23% -> 18%; README numbers updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/demo/Производитель А (демо)/Товар в пути (демо).xlsx
+++ b/data/demo/Производитель А (демо)/Товар в пути (демо).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:E13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,9 @@
       <c r="D1" t="str">
         <v>УТ-0001 от 15 сентября 2026 г. (поступление до 15.10.2026)</v>
       </c>
+      <c r="E1" t="str">
+        <v>Свободный остаток</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -426,6 +429,9 @@
       <c r="D2" t="str">
         <v/>
       </c>
+      <c r="E2">
+        <v>215</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -440,6 +446,9 @@
       <c r="D3">
         <v>1800</v>
       </c>
+      <c r="E3">
+        <v>453</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -454,6 +463,9 @@
       <c r="D4">
         <v>92</v>
       </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -468,6 +480,9 @@
       <c r="D5">
         <v>230</v>
       </c>
+      <c r="E5">
+        <v>119</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -482,6 +497,9 @@
       <c r="D6" t="str">
         <v/>
       </c>
+      <c r="E6">
+        <v>39</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -496,6 +514,9 @@
       <c r="D7">
         <v>138</v>
       </c>
+      <c r="E7">
+        <v>9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -510,6 +531,9 @@
       <c r="D8">
         <v>900</v>
       </c>
+      <c r="E8">
+        <v>29</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -524,6 +548,9 @@
       <c r="D9" t="str">
         <v/>
       </c>
+      <c r="E9">
+        <v>476</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -538,6 +565,9 @@
       <c r="D10" t="str">
         <v/>
       </c>
+      <c r="E10">
+        <v>15</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -552,6 +582,9 @@
       <c r="D11" t="str">
         <v/>
       </c>
+      <c r="E11">
+        <v>2148</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -566,6 +599,9 @@
       <c r="D12">
         <v>114</v>
       </c>
+      <c r="E12">
+        <v>53</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -580,10 +616,13 @@
       <c r="D13">
         <v>140</v>
       </c>
+      <c r="E13">
+        <v>63</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use source categories for seasonal demand; demo category effects A10 B8
Checks (30 days, growth 0): shield A q45/no-filter202/injected45; shield B q24/no-filter249/injected24. Cable A forecast2013/no-season2899; B1393/1905. Socket B q10/f175 versus no-stockout q0/f29. Category A DA0001 f445/q276 versus brand f416/q240; B DB0001 f238/q36 versus brand f218/q24. Real-data build: IEK776, Systeme205 rows.
</commit_message>
<xml_diff>
--- a/data/demo/Производитель А (демо)/Товар в пути (демо).xlsx
+++ b/data/demo/Производитель А (демо)/Товар в пути (демо).xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -415,6 +415,9 @@
       <c r="E1" t="str">
         <v>Свободный остаток</v>
       </c>
+      <c r="F1" t="str">
+        <v>Категория</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -432,6 +435,9 @@
       <c r="E2">
         <v>215</v>
       </c>
+      <c r="F2" t="str">
+        <v>Электроустановка</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -449,6 +455,9 @@
       <c r="E3">
         <v>453</v>
       </c>
+      <c r="F3" t="str">
+        <v>Кабель и монтаж</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -466,6 +475,9 @@
       <c r="E4">
         <v>0</v>
       </c>
+      <c r="F4" t="str">
+        <v>Освещение и защита</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -483,6 +495,9 @@
       <c r="E5">
         <v>119</v>
       </c>
+      <c r="F5" t="str">
+        <v>Электроустановка</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -500,6 +515,9 @@
       <c r="E6">
         <v>39</v>
       </c>
+      <c r="F6" t="str">
+        <v>Кабель и монтаж</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -517,6 +535,9 @@
       <c r="E7">
         <v>9</v>
       </c>
+      <c r="F7" t="str">
+        <v>Электроустановка</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -534,6 +555,9 @@
       <c r="E8">
         <v>29</v>
       </c>
+      <c r="F8" t="str">
+        <v>Электроустановка</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -551,6 +575,9 @@
       <c r="E9">
         <v>476</v>
       </c>
+      <c r="F9" t="str">
+        <v>Освещение и защита</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -568,6 +595,9 @@
       <c r="E10">
         <v>15</v>
       </c>
+      <c r="F10" t="str">
+        <v>Кабель и монтаж</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -585,6 +615,9 @@
       <c r="E11">
         <v>2148</v>
       </c>
+      <c r="F11" t="str">
+        <v>Кабель и монтаж</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -602,6 +635,9 @@
       <c r="E12">
         <v>53</v>
       </c>
+      <c r="F12" t="str">
+        <v>Освещение и защита</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -619,10 +655,13 @@
       <c r="E13">
         <v>63</v>
       </c>
+      <c r="F13" t="str">
+        <v>Освещение и защита</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>